<commit_message>
arreglo gafas para versiones anteriores y ptt permanente
</commit_message>
<xml_diff>
--- a/Seguimiento-IAM-AeriaOne.xlsx
+++ b/Seguimiento-IAM-AeriaOne.xlsx
@@ -712,7 +712,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>6 de septiembre de 2026 (actualizado al cerrar el workflow 3)</t>
+          <t>6 de septiembre de 2026; filas de los wf 4, 5, 30, 34, 46 y 61, IAM-16 y este recuento revisados el 15 de septiembre</t>
         </is>
       </c>
     </row>
@@ -780,12 +780,16 @@
         </is>
       </c>
       <c r="B17" s="10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C17" s="10" t="n">
-        <v>10.3</v>
-      </c>
-      <c r="D17" s="10" t="n"/>
+        <v>11.8</v>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>Completo por nuestra parte y verificado en dispositivo (Redmi Note 8 Pro, Samsung o W1)</t>
+        </is>
+      </c>
       <c r="E17" s="10" t="n"/>
       <c r="F17" s="10" t="inlineStr">
         <is>
@@ -800,10 +804,10 @@
         </is>
       </c>
       <c r="B18" s="10" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C18" s="10" t="n">
-        <v>33.8</v>
+        <v>35.3</v>
       </c>
       <c r="D18" s="10" t="n"/>
       <c r="E18" s="10" t="n"/>
@@ -820,10 +824,10 @@
         </is>
       </c>
       <c r="B19" s="10" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C19" s="10" t="n">
-        <v>30.9</v>
+        <v>27.9</v>
       </c>
       <c r="D19" s="10" t="n"/>
       <c r="E19" s="10" t="n"/>
@@ -1992,7 +1996,7 @@
       </c>
       <c r="M8" s="10" t="inlineStr">
         <is>
-          <t>Verificador REAL desde el 2026-09-06 y probado en el Redmi. El PIN no se guarda en ninguna forma: se guarda un testigo cifrado con AES-GCM bajo clave PBKDF2, y el fichero va envuelto ademas por una clave de Keystore PROPIA (distinta de la de evidencia, IAM-05). El contador de intentos sale de SharedPreferences en claro y entra en ese fichero sellado. Iteraciones CALIBRADAS midiendo el terminal (50.000 en el Redmi, 843 ms) en vez de copiadas: ver D8. Pantalla de alta con confirmacion y politica minima, 4 pruebas JVM. Falta ver en pantalla los rechazos y el bloqueo escalonado.</t>
+          <t>Verificador REAL desde el 2026-09-06 y probado en el Redmi. El PIN no se guarda en ninguna forma: se guarda un testigo cifrado con AES-GCM bajo clave PBKDF2, y el fichero va envuelto ademas por una clave de Keystore PROPIA (distinta de la de evidencia, IAM-05). El contador de intentos sale de SharedPreferences en claro y entra en ese fichero sellado. Iteraciones CALIBRADAS midiendo el terminal (50.000 en el Redmi, 843 ms) en vez de copiadas: ver D8. Pantalla de alta con confirmacion y politica minima, 4 pruebas JVM. Falta ver en pantalla los rechazos y el bloqueo escalonado. REVISADO el 2026-09-15 contra el codigo: sigue igual (desde el 06-sep solo cambio ClaveEnKeystore, sin efecto sobre el PIN) y el verificador conto como fallo un PIN mal tecleado en el Samsung. OJO: con SIMULADOR_CONFIANZA_EN_RELEASE=true la release de pruebas trae el simulador y el PIN 004471; quitarlo antes de auditar.</t>
         </is>
       </c>
     </row>
@@ -2027,11 +2031,11 @@
       </c>
       <c r="G9" s="12" t="inlineStr">
         <is>
-          <t>Sin empezar</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="H9" s="16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I9" s="9" t="inlineStr">
         <is>
@@ -2050,12 +2054,12 @@
       </c>
       <c r="L9" s="10" t="inlineStr">
         <is>
-          <t>data/identity/PinLocal.establecer()</t>
+          <t>feature/pinchange/ChangePinViewModel.kt, ChangePinScreen.kt, IdentityRepository.comprobarPinActual() y cambiarPin()</t>
         </is>
       </c>
       <c r="M9" s="10" t="inlineStr">
         <is>
-          <t>Cambio de PIN. Puramente local. Con el wf 4 cerrado ya no depende de nada: PinLocal.establecer() sustituye el verificador y reinicia el contador, solo falta la pantalla.</t>
+          <t>HECHO el 2026-09-15 y verificado en el Samsung. Profile &gt; Session &gt; Change PIN, en tres pasos: actual, nuevo y confirmacion. El actual se comprueba al teclearlo y cada fallo cuenta contra el MISMO limite que el desbloqueo: si no, un telefono perdido con la sesion abierta dejaria probar PINs sin limite. Agotar la tanda cierra la sesion. El nuevo pasa la politica del alta y tiene que ser distinto del actual. cambiarPin() vuelve a comprobar el actual antes de escribir el verificador. Prueba: PIN actual incorrecto -&gt; 'Wrong PIN. 4 attempts left'; cambio 004471 -&gt; 258036; tras bloquear, 004471 falla y 258036 abre. Sin verificar: el bloqueo por tanda agotada desde esta pantalla.</t>
         </is>
       </c>
     </row>
@@ -3606,7 +3610,7 @@
         </is>
       </c>
       <c r="H34" s="16" t="n">
-        <v>0.55</v>
+        <v>0.85</v>
       </c>
       <c r="I34" s="9" t="inlineStr">
         <is>
@@ -3625,12 +3629,12 @@
       </c>
       <c r="L34" s="10" t="inlineStr">
         <is>
-          <t>IdentityRepository.lock()</t>
+          <t>IdentityRepository.terminarTurno() y lock(motivo), AppContainer.alCerrarSesion, ProfileScreen (End shift)</t>
         </is>
       </c>
       <c r="M34" s="10" t="inlineStr">
         <is>
-          <t>Volver a bloqueado ya funciona y desde el 2026-09-06 ademas retira la autorizacion de la clave del agente, que era la mitad importante: sin eso la clave seguiria firmando con la pantalla bloqueada. Falta cerrar la sesion del servidor, deshacer bindings y sellar la boveda en el mismo gesto.</t>
+          <t>REVISADO el 2026-09-15: lock() existia pero ningun gesto la llamaba en uso normal (solo el reintentar de BLOCKED), asi que la sesion solo se cerraba si moria el proceso. HECHO ese dia: Profile &gt; Session &gt; End shift, con confirmacion y desactivado durante un SOS. Desata la bodycam con FIN_DE_TURNO, retira la autorizacion de la clave del agente, sella la boveda y borra las copias descifradas, y vuelve a LOCKED. Cualquier cierre de sesion sella ya la boveda. Verificado en el Samsung que bloquea y exige PIN. SIN VERIFICAR: desatar la bodycam y sellar una boveda configurada (el Samsung tiene identidad simulada y la boveda sin configurar; hay que probarlo con el Redmi y la W1). Lo que queda fuera es invalidar la sesion en el servidor, que es del backend.</t>
         </is>
       </c>
     </row>
@@ -3882,7 +3886,7 @@
       </c>
       <c r="M38" s="10" t="inlineStr">
         <is>
-          <t>Escrito el 2026-09-06: cerrar sesion deshace la atadura, y el fin va firmado igual que la creacion porque si cualquiera pudiera deshacerla bastaria acercarse a la camara para dejar al agente sin atribucion en mitad de un incidente. Caducidad comprobada al leer y no con temporizador (un temporizador que no salta deja una atadura viva de mas). Faltan los otros tres motivos del catalogo -reasignacion, revocacion y fin de turno explicito- y verificarlo en dispositivo.</t>
+          <t>Escrito el 2026-09-06: cerrar sesion deshace la atadura, y el fin va firmado igual que la creacion porque si cualquiera pudiera deshacerla bastaria acercarse a la camara para dejar al agente sin atribucion en mitad de un incidente. Caducidad comprobada al leer y no con temporizador (un temporizador que no salta deja una atadura viva de mas). Faltan los otros tres motivos del catalogo -reasignacion, revocacion y fin de turno explicito- y verificarlo en dispositivo. ACTUALIZADO el 2026-09-15: el fin de turno explicito ya existe (End shift manda FIN_DE_TURNO, que la W1 solo registra, sin cambios en BodyCamServer). Siguen faltando reasignacion y revocacion, y la verificacion en dispositivo sigue pendiente.</t>
         </is>
       </c>
     </row>
@@ -4614,7 +4618,7 @@
         </is>
       </c>
       <c r="H50" s="16" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="I50" s="9" t="inlineStr">
         <is>
@@ -4633,12 +4637,12 @@
       </c>
       <c r="L50" s="10" t="inlineStr">
         <is>
-          <t>feature/vault/VaultScreen.kt, ui/components/MediaPreview.kt</t>
+          <t>feature/vault/VaultScreen.kt, ui/components/MediaPreview.kt, VaultRepository.open() (auditoria), VaultViewModel</t>
         </is>
       </c>
       <c r="M50" s="10" t="inlineStr">
         <is>
-          <t>Visionado dentro de la app con contrasena y reproductor propio (el audio ya no sale a una app externa, que entregaba el claro a un tercero). Falta el permiso por politica y el evento de auditoria de quien miro.</t>
+          <t>Visionado dentro de la app con contrasena y reproductor propio (el audio ya no sale a una app externa, que entregaba el claro a un tercero). Falta el permiso por politica y el evento de auditoria de quien miro. ACTUALIZADO el 2026-09-15: el evento de auditoria ya existe. VaultRepository.open(), por donde pasan TODAS las vistas previas, registra EVIDENCIA_VISUALIZADA con el fichero y si llego a mostrarse; la boveda registra creada, abierta, contrasena incorrecta y cerrada (a mano o por fin de sesion). Sin verificar en telefono (el Samsung tiene la boveda sin configurar). Sigue faltando el permiso de visionado por politica.</t>
         </is>
       </c>
     </row>
@@ -5555,11 +5559,11 @@
       </c>
       <c r="G65" s="12" t="inlineStr">
         <is>
-          <t>Sin empezar</t>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="H65" s="16" t="n">
-        <v>0.1</v>
+        <v>0.6</v>
       </c>
       <c r="I65" s="9" t="inlineStr">
         <is>
@@ -5573,17 +5577,17 @@
       </c>
       <c r="K65" s="10" t="inlineStr">
         <is>
-          <t>Catalogo de eventos (G0)</t>
+          <t>Catalogo de eventos (G0): el nuestro es propuesta, falta que ciberseguridad lo ratifique</t>
         </is>
       </c>
       <c r="L65" s="10" t="inlineStr">
         <is>
-          <t>Log de Android, IncidentTimeline</t>
+          <t>data/audit/AuditoriaLocal.kt, CadenaDeAuditoria.kt, feature/audit/ (pantalla), CadenaDeAuditoriaTest</t>
         </is>
       </c>
       <c r="M65" s="10" t="inlineStr">
         <is>
-          <t>Hay trazas y timeline del incidente, pero no una cola de auditoria a prueba de manipulacion. El diario local se puede hacer entero sin backend.</t>
+          <t>HECHA LA MITAD CLIENTE el 2026-09-15, verificada en el Samsung. Diario local encadenado: cada evento lleva la HMAC-SHA256 del anterior con una clave PROPIA del Keystore (IAM-05), asi que cambiar, borrar de en medio, reordenar o renumerar rompe la cadena y rehacerla exige la clave. Campos del §14.1: id, hora, uptime (saltos de reloj), tipo, familia, agente, tenant, dispositivo, instancia, release y sesion; nunca contenido. Catalogo propuesto: sesion (abierta, PIN incorrecto, bloqueo, cambio de PIN, cerrada), periferico (enlace, atadura creada, rechazada, deshecha) y evidencia (boveda y visionado, wf 46). Profile &gt; Audit log muestra CHAIN INTACT o CHAIN BROKEN AT EVENT #N. 8 pruebas JVM, una por ataque. Prueba en telefono: evento #4 manipulado a mano -&gt; 'CHAIN BROKEN AT EVENT #4'. LIMITE: cortar el final no se detecta en local; solo el backend al recibir el diario. Falta: subida y correlacion (backend), rotacion y tope de tamano, y verificar los eventos de boveda y bodycam con el Redmi y la W1.</t>
         </is>
       </c>
     </row>
@@ -11682,7 +11686,7 @@
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>PIN real: verificador contra el Keystore, contador de intentos cifrado, alta y cambio</t>
+          <t>PIN real: verificador contra el Keystore, contador de intentos cifrado y alta con confirmacion. (El cambio de PIN es el wf 5, fila aparte.)</t>
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr">
@@ -11910,12 +11914,12 @@
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>Cola local de auditoria a prueba de manipulacion (encadenada por hash)</t>
+          <t>Diario local encadenado por HMAC con clave propia del Keystore y pantalla Audit log. Hecho el 2026-09-15; subirlo y correlarlo es del backend</t>
         </is>
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>Sin empezar</t>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="F11" s="10" t="inlineStr">
@@ -12024,7 +12028,7 @@
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>Cierre de turno completo: bloquear, deshacer bindings y sellar la boveda en un gesto</t>
+          <t>Fin de turno en un gesto (Profile &gt; End shift): desata la bodycam con FIN_DE_TURNO, retira la autorizacion de la clave del agente, sella la boveda y bloquea. Hecho el 2026-09-15; falta verificar desatar y sellar con el Redmi y la W1, y la sesion del servidor es del backend</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
@@ -12044,7 +12048,7 @@
       </c>
       <c r="H14" s="10" t="inlineStr">
         <is>
-          <t>Bloquear y sellar ya existen por separado; falta unirlos y anadir el aviso.</t>
+          <t>Todo el gesto es local. Lo unico que no es nuestro es invalidar la sesion en el servidor, que hoy no existe.</t>
         </is>
       </c>
     </row>
@@ -12062,12 +12066,12 @@
       </c>
       <c r="D15" s="10" t="inlineStr">
         <is>
-          <t>Cambio de PIN</t>
+          <t>Cambio de PIN en Profile: actual, nuevo y confirmacion; los fallos cuentan contra el limite del desbloqueo. Hecho el 2026-09-15</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Sin empezar</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F15" s="10" t="inlineStr">
@@ -12176,7 +12180,7 @@
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>Registro de auditoria de quien abre la boveda y que evidencia mira</t>
+          <t>Evento de auditoria de quien abre la boveda y que evidencia mira: hecho el 2026-09-15. Falta el permiso de visionado por politica</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
@@ -13030,10 +13034,10 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B31:E31"/>
+    <mergeCell ref="B26:E26"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="B26:E26"/>
     <mergeCell ref="B27:E27"/>
-    <mergeCell ref="B31:E31"/>
     <mergeCell ref="B35:E35"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B30:E30"/>
@@ -13191,7 +13195,7 @@
       </c>
       <c r="F7" s="12" t="inlineStr">
         <is>
-          <t>Sin empezar</t>
+          <t>Parcial (propuesta nuestra en AuditoriaLocal.TipoEvento, sin ratificar)</t>
         </is>
       </c>
     </row>
@@ -13779,7 +13783,7 @@
       </c>
       <c r="F28" s="11" t="inlineStr">
         <is>
-          <t>Parcial (boveda hecha)</t>
+          <t>Parcial (evento de auditoria hecho; falta permiso por politica)</t>
         </is>
       </c>
     </row>
@@ -14115,7 +14119,7 @@
       </c>
       <c r="F40" s="12" t="inlineStr">
         <is>
-          <t>Sin empezar</t>
+          <t>Hecho (2026-09-15)</t>
         </is>
       </c>
     </row>
@@ -15813,7 +15817,7 @@
       </c>
       <c r="C20" s="12" t="inlineStr">
         <is>
-          <t>Sin empezar</t>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="D20" s="10" t="inlineStr">
@@ -15823,7 +15827,7 @@
       </c>
       <c r="E20" s="10" t="inlineStr">
         <is>
-          <t>Hay trazas, no auditoria.</t>
+          <t>Diario local a prueba de manipulacion desde el 2026-09-15 (wf 61), con eventos de sesion, periferico y evidencia. Falta correlarlo con el servidor, que es del backend.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cifrado con bluetooth con la bodycam
</commit_message>
<xml_diff>
--- a/Seguimiento-IAM-AeriaOne.xlsx
+++ b/Seguimiento-IAM-AeriaOne.xlsx
@@ -8,21 +8,22 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalogo-68" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detalle-pasos" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sin-backend-YA" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bloqueado-backend" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan-G0-G7" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Septiembre-2026" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisiones" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requisitos-IAM" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deuda-hallazgos" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflows" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalogo-68" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detalle-pasos" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sin-backend-YA" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bloqueado-backend" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan-G0-G7" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Septiembre-2026" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisiones" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requisitos-IAM" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deuda-hallazgos" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Catalogo-68'!$A$4:$M$72</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Detalle-pasos'!$A$4:$G$166</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Plan-G0-G7'!$A$4:$F$49</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Deuda-hallazgos'!$A$4:$G$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Catalogo-68'!$A$4:$M$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Detalle-pasos'!$A$4:$G$166</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Plan-G0-G7'!$A$4:$F$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Deuda-hallazgos'!$A$4:$G$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -31,7 +32,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -90,8 +91,60 @@
       <color rgb="001F3864"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <color rgb="0044546A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00595959"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00006100"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="009C0006"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="009C5700"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -128,8 +181,25 @@
         <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDEDED"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -195,11 +265,16 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -257,6 +332,65 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -332,6 +466,32 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:D69" headerRowCount="1">
+  <autoFilter ref="A1:D69"/>
+  <tableColumns count="4">
+    <tableColumn id="1" name="#"/>
+    <tableColumn id="2" name="Workflow"/>
+    <tableColumn id="3" name="Purpose"/>
+    <tableColumn id="4" name="Status"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Revision" displayName="Revision" ref="F1:I69" headerRowCount="1">
+  <autoFilter ref="F1:I69"/>
+  <tableColumns count="4">
+    <tableColumn id="6" name="App movil"/>
+    <tableColumn id="7" name="Detalle app movil"/>
+    <tableColumn id="8" name="Bodycam"/>
+    <tableColumn id="9" name="Detalle bodycam"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1195,6 +1355,636 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00ED7D31"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="62" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="74" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Trazabilidad de los requisitos IAM-01 a IAM-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="26" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Apartado 15 del documento de arquitectura, contrastado contra el codigo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Requisito</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Cobertura hoy</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>Workflows implicados</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>Nota</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>IAM-01</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Identidad unica y autoritativa para tenant, usuario, dispositivo, credencial, release, instancia de APK, workload, sesion y evidencia</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>12, 23, 36</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>Dispositivo: si, DEV-8DB2C628 real. Instancia de APK: valor de demo. Evidencia: hay identificador, falta manifiesto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>IAM-02</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Datos, politica y administracion de QPD aislados de otros tenants</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>Backend.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>IAM-03</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>El acceso rutinario recupera el usuario ya enlazado y usa la clave protegida autorizada por PIN</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>4, 27</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>La pantalla NO pide usuario y el PIN autoriza de verdad el uso de la clave: sin el, firmar como el agente es un error de programacion y no una posibilidad. Lo que falta es que esa autorizacion sea del KEYSTORE y no de la app, que es la decision D2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>IAM-04</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Reto-respuesta fresco; ni el PIN ni la clave privada se transmiten</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Cumplido en el cliente</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>12, 3, 27</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>La clave nunca sale del Keystore y el PIN tampoco viaja. Desde el 2026-09-06 los cinco puntos que firman usan un nonce ajeno, de un solo uso y con caducidad, verificado con openssl; repetir una respuesta se rechaza. Lo unico que falta para cumplirlo del todo no es del cliente: que el emisor sea un backend y no tools/reto.sh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>IAM-05</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Claves separadas por proposito e independientemente revocables para usuario, dispositivo, aplicacion y evidencia</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>3, 12, 37, 38</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>Dispositivo y evidencia ya estan separadas. Falta la del agente (wf 3) y la de firma de evidencia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="15" t="inlineStr">
+        <is>
+          <t>IAM-06</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>El registro de relaciones es autoritativo para las relaciones y su historia</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>23, 33, 34</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>El registro autoritativo es del backend y no existe. Lo que si hay desde el 2026-09-06 es la relacion agente-periferico como declaracion firmada con caducidad, que es la mitad que se puede sostener desde el cliente. Falta la atadura agente-telefono registrada (wf 23) y toda la historia de las relaciones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>IAM-07</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Solo releases aprobados e instancias activas y enlazadas llegan a produccion</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>21, 22, 23, 25</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>Hoy cualquier APK instalado arranca.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="15" t="inlineStr">
+        <is>
+          <t>IAM-08</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>La autorizacion evalua tenant, sujeto, dispositivos, software, bindings, permisos, recurso, accion y contexto</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>Backend. El cliente aun decide en local.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>IAM-09</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Sesiones cortas, con alcance, identificables y terminables</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>28, 29, 30</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>No hay token de sesion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>IAM-10</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>Los perifericos mantienen identidad propia y nunca suplantan al agente</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>13, 31, 33</t>
+        </is>
+      </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>Verificado sobre hardware el 2026-09-06: la W1 tiene par de claves propio en su Keystore (BWC-896E) y el canal lleva reto-respuesta mutuo. La camara es un tercer sujeto de confianza que se revoca por su lado, no una extension del telefono. Falta el binding agente-camara con caducidad (wf 33).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>IAM-11</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>La evidencia tiene procedencia verificable, integridad, cifrado y custodia</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>36, 37, 38, 42</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="inlineStr">
+        <is>
+          <t>Cifrado y custodia local: hechos. Procedencia y firma: pendientes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>IAM-12</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>La aceptacion del servidor precede al borrado local controlado por politica</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>44, 45</t>
+        </is>
+      </c>
+      <c r="E16" s="10" t="inlineStr">
+        <is>
+          <t>El recibo lo escribe hoy el propio telefono.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>IAM-13</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>La autorizacion offline es firmada, acotada y reconciliada</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>50, 51, 52</t>
+        </is>
+      </c>
+      <c r="E17" s="10" t="inlineStr">
+        <is>
+          <t>Hoy todo funciona offline sin gobierno: es el hueco mas grande respecto al modelo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="15" t="inlineStr">
+        <is>
+          <t>IAM-14</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Revocacion granular sobre todos los sujetos de confianza</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>8, 16, 26, 60</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t>Los 9 interruptores del §13 estan modelados en TrustBlockReason; falta el canal. Choca con la boveda (D5).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>IAM-15</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>La revocacion preserva la atribucion historica del momento de la firma</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="inlineStr">
+        <is>
+          <t>Requiere firma de evidencia (wf 37).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>IAM-16</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>Eventos de seguridad, administracion, autorizacion y evidencia correlados y a prueba de manipulacion</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>Diario local a prueba de manipulacion desde el 2026-09-15 (wf 61), con eventos de sesion, periferico y evidencia. Falta correlarlo con el servidor, que es del backend.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>IAM-17</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>Los workloads del backend usan identidades propias de minimo privilegio</t>
+        </is>
+      </c>
+      <c r="C21" s="12" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="D21" s="10" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="E21" s="10" t="inlineStr">
+        <is>
+          <t>Backend.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>IAM-18</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>Reseteo o reparacion exigen nueva alta y vuelta a servicio</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="D22" s="10" t="inlineStr">
+        <is>
+          <t>66, 67</t>
+        </is>
+      </c>
+      <c r="E22" s="10" t="inlineStr">
+        <is>
+          <t>La clave se destruye con el reseteo, pero no se DETECTA: la app simplemente deja de funcionar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
+          <t>IAM-19</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>La rotacion de CA admite solape controlado y migracion de la flota</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="D23" s="10" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="E23" s="10" t="inlineStr">
+        <is>
+          <t>Hoy solo hay una CA de pruebas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="15" t="inlineStr">
+        <is>
+          <t>IAM-20</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>La linea base no reclama biometria ni MFA formal para el agente</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Cumplido</t>
+        </is>
+      </c>
+      <c r="D24" s="10" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="E24" s="10" t="inlineStr">
+        <is>
+          <t>La app no usa biometria. Coherente por diseno, no por omision.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="20" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B26" s="21" t="inlineStr">
+        <is>
+          <t>20 requisitos</t>
+        </is>
+      </c>
+      <c r="C26" s="21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D26" s="21" t="inlineStr">
+        <is>
+          <t>Cumplido: 1 | Parcial: 9 | Sin empezar: 7 | No aplica (backend): 2</t>
+        </is>
+      </c>
+      <c r="E26" s="21" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="00C00000"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -1643,6 +2433,2880 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M69"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4.140625" customWidth="1" min="1" max="1"/>
+    <col width="43.85546875" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13.5703125" customWidth="1" min="4" max="4"/>
+    <col width="3" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="39" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="39" t="inlineStr">
+        <is>
+          <t>Workflow</t>
+        </is>
+      </c>
+      <c r="C1" s="39" t="inlineStr">
+        <is>
+          <t>Purpose</t>
+        </is>
+      </c>
+      <c r="D1" s="39" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>App movil</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Detalle app movil</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Bodycam</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Detalle bodycam</t>
+        </is>
+      </c>
+      <c r="K1" s="28" t="inlineStr">
+        <is>
+          <t>Recuento</t>
+        </is>
+      </c>
+      <c r="L1" s="28" t="inlineStr">
+        <is>
+          <t>App movil</t>
+        </is>
+      </c>
+      <c r="M1" s="28" t="inlineStr">
+        <is>
+          <t>Bodycam</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="41" t="inlineStr">
+        <is>
+          <t>Tenant / Organization Onboarding</t>
+        </is>
+      </c>
+      <c r="C2" s="40" t="inlineStr">
+        <is>
+          <t>Create QPD tenant, CA trust, policies, roles, admins</t>
+        </is>
+      </c>
+      <c r="F2" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>Alta del tenant: backend / QPD.</t>
+        </is>
+      </c>
+      <c r="H2" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2" s="31" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="L2">
+        <f>COUNTIF(Revision[App movil],K2)</f>
+        <v/>
+      </c>
+      <c r="M2">
+        <f>COUNTIF(Revision[Bodycam],K2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="43" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="44" t="inlineStr">
+        <is>
+          <t>User Enrollment</t>
+        </is>
+      </c>
+      <c r="C3" s="43" t="inlineStr">
+        <is>
+          <t>Create cmendez.aeriaone.com, assign QPD, role and entitlements</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="F3" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>Los 10 pasos son de administrador; la app hereda la identidad ya creada.</t>
+        </is>
+      </c>
+      <c r="H3" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K3" s="32" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="L3">
+        <f>COUNTIF(Revision[App movil],K3)</f>
+        <v/>
+      </c>
+      <c r="M3">
+        <f>COUNTIF(Revision[Bodycam],K3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="43" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="44" t="inlineStr">
+        <is>
+          <t>User Certificate Issuance</t>
+        </is>
+      </c>
+      <c r="C4" s="43" t="inlineStr">
+        <is>
+          <t>Generate hardware-backed key, CSR, issue and bind user certificate</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="F4" s="45" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Par EC P-256 del agente en el TEE, CSR contrafirmado por el terminal. Desde el 18-sep el certificado lo emite el IAM real (iam/users/enroll); verificado en el Samsung contra el backend local. CredentialRepository.kt.</t>
+        </is>
+      </c>
+      <c r="H4" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K4" s="34" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="L4">
+        <f>COUNTIF(Revision[App movil],K4)</f>
+        <v/>
+      </c>
+      <c r="M4">
+        <f>COUNTIF(Revision[Bodycam],K4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="44" t="inlineStr">
+        <is>
+          <t>User PIN / Password Setup</t>
+        </is>
+      </c>
+      <c r="C5" s="43" t="inlineStr">
+        <is>
+          <t>Establish local secret protecting use of the user credential/key</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="F5" s="45" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>PIN con verificador real (PBKDF2 + AES-GCM sellado por clave de Keystore propia), iteraciones calibradas. PinLocal.kt. Abierto: D1, D2, D8.</t>
+        </is>
+      </c>
+      <c r="H5" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K5" s="35" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="L5">
+        <f>COUNTIF(Revision[App movil],K5)</f>
+        <v/>
+      </c>
+      <c r="M5">
+        <f>COUNTIF(Revision[Bodycam],K5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="40" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="41" t="inlineStr">
+        <is>
+          <t>User PIN / Password Change</t>
+        </is>
+      </c>
+      <c r="C6" s="40" t="inlineStr">
+        <is>
+          <t>Normal credential change</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F6" s="45" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Profile &gt; Change PIN, con el mismo limite de intentos que el desbloqueo. Verificado en el Samsung el 15-sep. feature/pinchange/.</t>
+        </is>
+      </c>
+      <c r="H6" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K6" s="36" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="L6" s="36">
+        <f>SUM(L2:L5)</f>
+        <v/>
+      </c>
+      <c r="M6" s="36">
+        <f>SUM(M2:M5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="40" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="41" t="inlineStr">
+        <is>
+          <t>Forgotten PIN / Password Recovery</t>
+        </is>
+      </c>
+      <c r="C7" s="40" t="inlineStr">
+        <is>
+          <t>Controlled recovery/re-enrollment without weakening PKI trust</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F7" s="46" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Nada. Necesita re-alta autorizada por el backend.</t>
+        </is>
+      </c>
+      <c r="H7" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="47" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="48" t="inlineStr">
+        <is>
+          <t>User Certificate Renewal</t>
+        </is>
+      </c>
+      <c r="C8" s="47" t="inlineStr">
+        <is>
+          <t>Replace certificate approaching expiry while retaining identity</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Needs Rework</t>
+        </is>
+      </c>
+      <c r="F8" s="46" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Nada. Ciber lo marca Needs Rework.</t>
+        </is>
+      </c>
+      <c r="H8" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K8" s="49" t="inlineStr">
+        <is>
+          <t>Revisado contra el codigo el 25-sep-2026 (app dev_back_connection 009c548, BodyCamServer dev_install_assistant cb6a247) y actualizado esa tarde con los cambios sin commitear: compilan, pero NO estan probados en dispositivo, asi que ninguno pasa a Hecho.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="40" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="41" t="inlineStr">
+        <is>
+          <t>User Certificate Revocation</t>
+        </is>
+      </c>
+      <c r="C9" s="40" t="inlineStr">
+        <is>
+          <t>Immediately invalidate compromised/terminated/suspended identity</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F9" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>El corte existe (TrustBlockReason.CERTIFICATE_REVOKED); falta el canal que lo dispare.</t>
+        </is>
+      </c>
+      <c r="H9" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>La camara no consulta revocaciones del agente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="40" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="41" t="inlineStr">
+        <is>
+          <t>User Suspension / Reactivation</t>
+        </is>
+      </c>
+      <c r="C10" s="40" t="inlineStr">
+        <is>
+          <t>Temporarily disable backend authorization without necessarily destroying identity</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F10" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Estado USER_DISABLED modelado; falta el emisor.</t>
+        </is>
+      </c>
+      <c r="H10" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="40" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="41" t="inlineStr">
+        <is>
+          <t>User Offboarding</t>
+        </is>
+      </c>
+      <c r="C11" s="40" t="inlineStr">
+        <is>
+          <t>Revoke credentials, terminate bindings/sessions and remove entitlements</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F11" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Baja del agente: backend / QPD.</t>
+        </is>
+      </c>
+      <c r="H11" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="43" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="44" t="inlineStr">
+        <is>
+          <t>Device Manufacturing Enrollment</t>
+        </is>
+      </c>
+      <c r="C12" s="43" t="inlineStr">
+        <is>
+          <t>Establish immutable device identity and device certificate</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="F12" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>Alta de fabrica.</t>
+        </is>
+      </c>
+      <c r="H12" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>D4: la W1 no puede pasar por el alta de fabrica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="40" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="41" t="inlineStr">
+        <is>
+          <t>Android Mobile Device Enrollment</t>
+        </is>
+      </c>
+      <c r="C13" s="40" t="inlineStr">
+        <is>
+          <t>Register Android/phone, attest hardware, issue device identity</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F13" s="45" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>Par EC en el TEE con atestacion y PKCS#10. Desde el 18-sep contra el IAM real (iam/devices/enroll): el telefono adopta el device_id del backend. Verificado en el Samsung (DEV-6B85FB5C).</t>
+        </is>
+      </c>
+      <c r="H13" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="40" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="41" t="inlineStr">
+        <is>
+          <t>Body Camera Enrollment</t>
+        </is>
+      </c>
+      <c r="C14" s="40" t="inlineStr">
+        <is>
+          <t>Establish independent BWC identity and certificate</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F14" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Solo guarda el ancla de perifericos, que sigue siendo la CA de pruebas por adb (el backend ya devuelve la suya).</t>
+        </is>
+      </c>
+      <c r="H14" s="45" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>Par EC P-256 en el Keystore de la W1, CSR BWC-896E y certificado de la Device CA. Verificado el 06-sep. OJO: con tools/alta-bodycam.sh y la CA de pruebas, no contra el IAM real. BodycamIdentity.kt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="40" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="41" t="inlineStr">
+        <is>
+          <t>Smart Goggles Enrollment</t>
+        </is>
+      </c>
+      <c r="C15" s="40" t="inlineStr">
+        <is>
+          <t>Establish independent goggles identity and certificate</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F15" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Hay gafas FalconOne desde el 13-sep, pero su firmware es del fabricante: no podemos generar clave en ellas.</t>
+        </is>
+      </c>
+      <c r="H15" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="40" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="41" t="inlineStr">
+        <is>
+          <t>Device Certificate Renewal</t>
+        </is>
+      </c>
+      <c r="C16" s="40" t="inlineStr">
+        <is>
+          <t>Rotate expiring device certificates</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F16" s="46" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>Nada. El cliente reutilizaria el codigo del wf 12.</t>
+        </is>
+      </c>
+      <c r="H16" s="46" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>Nada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="40" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="41" t="inlineStr">
+        <is>
+          <t>Device Certificate Revocation</t>
+        </is>
+      </c>
+      <c r="C17" s="40" t="inlineStr">
+        <is>
+          <t>Revoke compromised/lost/decommissioned device</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F17" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>Estado DEVICE_REVOKED modelado y visible; falta el canal.</t>
+        </is>
+      </c>
+      <c r="H17" s="46" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>La camara no tiene estado de revocacion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="40" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="41" t="inlineStr">
+        <is>
+          <t>Device Reassignment</t>
+        </is>
+      </c>
+      <c r="C18" s="40" t="inlineStr">
+        <is>
+          <t>Move device from one officer/unit to another safely</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F18" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>Registro de dispositivos: backend / QPD.</t>
+        </is>
+      </c>
+      <c r="H18" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="40" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="41" t="inlineStr">
+        <is>
+          <t>Device Replacement</t>
+        </is>
+      </c>
+      <c r="C19" s="40" t="inlineStr">
+        <is>
+          <t>Replace failed/damaged device while preserving administrative continuity</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F19" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>Registro de dispositivos: backend / QPD.</t>
+        </is>
+      </c>
+      <c r="H19" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="40" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="41" t="inlineStr">
+        <is>
+          <t>Lost / Stolen Device</t>
+        </is>
+      </c>
+      <c r="C20" s="40" t="inlineStr">
+        <is>
+          <t>Revoke trust, terminate bindings/sessions, quarantine and optionally wipe</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F20" s="46" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>Nada: ni cuarentena ni borrado remoto.</t>
+        </is>
+      </c>
+      <c r="H20" s="46" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>Nada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="40" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="41" t="inlineStr">
+        <is>
+          <t>Device Decommissioning</t>
+        </is>
+      </c>
+      <c r="C21" s="40" t="inlineStr">
+        <is>
+          <t>Revoke certificate, destroy keys, wipe and retire inventory</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F21" s="46" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>Nada propio (deshacerAlta() existe solo como reset de pruebas).</t>
+        </is>
+      </c>
+      <c r="H21" s="46" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>Nada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="43" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="44" t="inlineStr">
+        <is>
+          <t>APK Build &amp; Release</t>
+        </is>
+      </c>
+      <c r="C22" s="43" t="inlineStr">
+        <is>
+          <t>CI/CD → scan → approve → AeriaOne production signing</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="F22" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>Compilacion, versionado verificado con aapt2 y firma. Faltan SAST, SCA, secretos, SBOM y registro del artefacto.</t>
+        </is>
+      </c>
+      <c r="H22" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>Firma release propia (signingConfigs). Sin SAST, SCA ni registro del artefacto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="47" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="48" t="inlineStr">
+        <is>
+          <t>APK Initial Installation</t>
+        </is>
+      </c>
+      <c r="C23" s="47" t="inlineStr">
+        <is>
+          <t>Controlled distribution and installation</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Needs Rework</t>
+        </is>
+      </c>
+      <c r="F23" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>TrustGate en el primer arranque; falta verificar firma e integridad del artefacto.</t>
+        </is>
+      </c>
+      <c r="H23" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>Rama dev_device_owner/dev_install_assistant (20-24 sep): la app como device owner y lanzador, aprovisionada por tools/kiosco.sh. Es control de la unidad, no distribucion controlada. Asistente de instalacion en primer intento, sin verificar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="47" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="48" t="inlineStr">
+        <is>
+          <t>APK Activation / User Binding</t>
+        </is>
+      </c>
+      <c r="C24" s="47" t="inlineStr">
+        <is>
+          <t>Validate APK + device + cmendez.aeriaone.com + entitlement</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Needs Rework</t>
+        </is>
+      </c>
+      <c r="F24" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>La relacion agente &lt;-&gt; terminal la registra el backend en el alta. 25-sep (sin probar): app_instance_id propio por instalacion (APPINST- + 16 hex aleatorios) en noBackupFilesDir, en vez de la constante APPINST-8F27A91C comun a todos los telefonos; reinstalar o deshacer el alta da otra. Falta atarla a la release aprobada. Deuda: allowBackup=true lleva las preferencias a la copia de Google.</t>
+        </is>
+      </c>
+      <c r="H24" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="40" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="41" t="inlineStr">
+        <is>
+          <t>APK Update</t>
+        </is>
+      </c>
+      <c r="C25" s="40" t="inlineStr">
+        <is>
+          <t>Authenticate and securely install approved application version</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F25" s="46" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>Nada.</t>
+        </is>
+      </c>
+      <c r="H25" s="46" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
+          <t>Nada (se actualiza por adb install).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="40" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="41" t="inlineStr">
+        <is>
+          <t>APK Rollback Prevention</t>
+        </is>
+      </c>
+      <c r="C26" s="40" t="inlineStr">
+        <is>
+          <t>Prevent installation/use of vulnerable or unauthorized versions</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F26" s="46" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>Nada en cliente. La app ya manda app_version al abrir sesion, asi que el backend podria rechazarla.</t>
+        </is>
+      </c>
+      <c r="H26" s="46" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>Nada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="40" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="41" t="inlineStr">
+        <is>
+          <t>APK Revocation / Kill</t>
+        </is>
+      </c>
+      <c r="C27" s="40" t="inlineStr">
+        <is>
+          <t>Backend blocks a compromised/deprecated application release</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F27" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>Estado RELEASE_REVOKED modelado; app_version viaja en iam/session. Falta que el rechazo llegue a la pantalla de bloqueo.</t>
+        </is>
+      </c>
+      <c r="H27" s="46" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="I27" s="5" t="inlineStr">
+        <is>
+          <t>Nada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="40" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="41" t="inlineStr">
+        <is>
+          <t>User Login / Unlock</t>
+        </is>
+      </c>
+      <c r="C28" s="40" t="inlineStr">
+        <is>
+          <t>PIN/password unlocks use of the already provisioned user identity</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F28" s="45" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>PIN -&gt; reto de iam/challenge -&gt; firma con la clave del agente -&gt; sesion ACREDITADA. Verificado en el Samsung contra el backend el 18-sep. El PIN no espera a la red (SOLO_LOCAL hasta acreditarse). 25-sep (sin probar): si no hay red al desbloquear se reintenta solo (30 s, 1, 2 y 5 min), antes no se reintentaba nunca.</t>
+        </is>
+      </c>
+      <c r="H28" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="40" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="41" t="inlineStr">
+        <is>
+          <t>Session Establishment</t>
+        </is>
+      </c>
+      <c r="C29" s="40" t="inlineStr">
+        <is>
+          <t>Backend validates user + device + APK + tenant + authorization</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F29" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>Cliente hecho: iam/session con reto firmado, device_id, app_instance_id y app_version; token solo en memoria (SesionBackend) y usado en subidas y SOS. 25-sep: el token se presta tambien a la W1. Falta: app_instance_id real y hacerlo sin el tunel adb.</t>
+        </is>
+      </c>
+      <c r="H29" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="I29" s="5" t="inlineStr">
+        <is>
+          <t>25-sep (sin probar): usa el token de la sesion del AGENTE que le presta el telefono (TOKEN:&lt;jwt&gt;:&lt;segundos&gt;), solo de un telefono acreditado y solo en memoria. Decision del usuario para la demo: la unidad lleva todos los alcances del agente, por RFCOMM sin cifrar, y en el backend sube como el terminal del agente. Sin sesion propia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="40" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="41" t="inlineStr">
+        <is>
+          <t>Session Renewal</t>
+        </is>
+      </c>
+      <c r="C30" s="40" t="inlineStr">
+        <is>
+          <t>Safely refresh short-lived authorization/session tokens</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F30" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>25-sep (sin probar): IdentityRepository.mantenerAcreditada renueva 10 min antes de caducar abriendo otra sesion (no hay endpoint de renovacion) y cierra el token anterior. Si caduca sin renovar, vuelve a SOLO_LOCAL a la vista.</t>
+        </is>
+      </c>
+      <c r="H30" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="I30" s="5" t="inlineStr">
+        <is>
+          <t>25-sep (sin probar): recibe cada token renovado del telefono y TOKEN_CLEAR si caduca. Depende del telefono.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="40" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="41" t="inlineStr">
+        <is>
+          <t>Logout / Session Termination</t>
+        </is>
+      </c>
+      <c r="C31" s="40" t="inlineStr">
+        <is>
+          <t>Terminate operational session and temporary bindings</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F31" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>Profile &gt; End shift: bloquea, retira la autorizacion de la clave, sella la boveda, manda FIN_DE_TURNO e invalida el token en iam/session/logout. 25-sep: tambien para la renovacion y manda TOKEN_CLEAR a la W1. Falta verificar con el Redmi y la W1 el desatado y la boveda configurada.</t>
+        </is>
+      </c>
+      <c r="H31" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="inlineStr">
+        <is>
+          <t>Recibe FIN_DE_TURNO y solo lo registra. 25-sep: TOKEN_CLEAR retira el token prestado y el UNBIND suelta al agente rotulado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="40" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="41" t="inlineStr">
+        <is>
+          <t>Android ↔ Body Camera Pairing</t>
+        </is>
+      </c>
+      <c r="C32" s="40" t="inlineStr">
+        <is>
+          <t>Mutually authenticate devices and establish secure relationship</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F32" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>Reto-respuesta mutuo verificado sobre la W1 el 06-sep. Falta cifrar el canal y cortar los enlaces no autenticados (hoy solo se marcan). 25-sep: el token de sesion solo se manda por un enlace autenticado.</t>
+        </is>
+      </c>
+      <c r="H32" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="I32" s="5" t="inlineStr">
+        <is>
+          <t>Contraparte del reto-respuesta, verificada. OJO: pese al commit 'cifrado de conexion con bodycam' (c65bd1c), el canal NO va cifrado, y la camara acepta REC_*/SOS de un telefono sin acreditar: solo BIND y TOKEN exigen acreditacion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="40" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="41" t="inlineStr">
+        <is>
+          <t>Android ↔ Goggles Pairing</t>
+        </is>
+      </c>
+      <c r="C33" s="40" t="inlineStr">
+        <is>
+          <t>Same for smart goggles</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F33" s="46" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>Gafas conectadas desde el 13-sep con el SDK del fabricante y MAC elegida en la app, sin autenticacion nuestra. Mutua solo si el fabricante lo permite.</t>
+        </is>
+      </c>
+      <c r="H33" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="I33" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="40" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="41" t="inlineStr">
+        <is>
+          <t>Officer ↔ Peripheral Binding</t>
+        </is>
+      </c>
+      <c r="C34" s="40" t="inlineStr">
+        <is>
+          <t>Temporarily associate BWC/goggles operation with cmendez.aeriaone.com</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F34" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>BindingPeriferico.kt: atadura firmada con la clave del agente, 12 h, atada al nonce. 25-sep: la declaracion firmada lleva ademas nombre, rango y placa. SIN VERIFICAR en dispositivo; de ella dependen ya el token y el nombre de la W1.</t>
+        </is>
+      </c>
+      <c r="H34" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="I34" s="5" t="inlineStr">
+        <is>
+          <t>BindingAgente.kt comprueba CA de usuario, firma, camara, sesion y CN. 25-sep: la vigencia se cuenta con el reloj de la W1 (duracion firmada) y no con la hora del telefono; al atar, AgenteDeServicio guarda el agente que se rotula. SIN VERIFICAR en dispositivo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="40" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="41" t="inlineStr">
+        <is>
+          <t>Peripheral Unbinding</t>
+        </is>
+      </c>
+      <c r="C35" s="40" t="inlineStr">
+        <is>
+          <t>Shift end, logout, timeout, reassignment or revocation</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F35" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>Fin firmado por cierre de sesion y fin de turno. Faltan reasignacion y revocacion, y verificar en dispositivo.</t>
+        </is>
+      </c>
+      <c r="H35" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="I35" s="5" t="inlineStr">
+        <is>
+          <t>Deshacer firmado y caducidad al leer. 25-sep: deshacer, caducar o perder el enlace suelta al agente rotulado. Sin verificar en dispositivo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="40" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="41" t="inlineStr">
+        <is>
+          <t>Recording Start Authorization</t>
+        </is>
+      </c>
+      <c r="C36" s="40" t="inlineStr">
+        <is>
+          <t>Establish authenticated officer/device/session context before recording</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F36" s="46" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>Se graba sin comprobar sesion ni atadura.</t>
+        </is>
+      </c>
+      <c r="H36" s="46" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="I36" s="5" t="inlineStr">
+        <is>
+          <t>Graba sin atadura. 25-sep: sin agente atado el video sale UNASSIGNED en vez de John Smith, pero grabar sigue sin exigir nada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="40" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="41" t="inlineStr">
+        <is>
+          <t>Evidence Creation</t>
+        </is>
+      </c>
+      <c r="C37" s="40" t="inlineStr">
+        <is>
+          <t>Create video/photo/audio with provenance metadata</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F37" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>Captura verificada + manifiesto phone-incident/1 desde el 18-sep (agente, ubicacion real, linea de tiempo, sha256 y tipo). Faltan tenant, device_id, instancia, sesion y hora fiable.</t>
+        </is>
+      </c>
+      <c r="H37" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="I37" s="5" t="inlineStr">
+        <is>
+          <t>25-sep (sin probar): fuera HardcodedOfficer. Cada incidente congela al empezar el agente atado en officer.json; de ahi salen el manifiesto (con officer_user_id), los nombres de fichero, el rotulo del proxy y la subida. Sin agente: UNASSIGNED.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="40" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="41" t="inlineStr">
+        <is>
+          <t>Evidence Signing</t>
+        </is>
+      </c>
+      <c r="C38" s="40" t="inlineStr">
+        <is>
+          <t>Cryptographically sign artefact/hash and associated provenance</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F38" s="46" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>Solo hash SHA-256 en la cabecera FEVD: integridad, no origen.</t>
+        </is>
+      </c>
+      <c r="H38" s="46" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="I38" s="5" t="inlineStr">
+        <is>
+          <t>Igual: hash sin firma.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="40" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="41" t="inlineStr">
+        <is>
+          <t>Evidence Encryption</t>
+        </is>
+      </c>
+      <c r="C39" s="40" t="inlineStr">
+        <is>
+          <t>Encrypt artefact using evidence-specific encryption scheme</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F39" s="45" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>FEVD v1: AES-GCM por bloques, DEK envuelta con RSA-OAEP a boveda + Nexus. EvidenceCrypto.kt.</t>
+        </is>
+      </c>
+      <c r="H39" s="45" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I39" s="5" t="inlineStr">
+        <is>
+          <t>Mismo formato FEVD v1. EvidenceCrypto.kt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="41" t="inlineStr">
+        <is>
+          <t>Evidence Local Storage</t>
+        </is>
+      </c>
+      <c r="C40" s="40" t="inlineStr">
+        <is>
+          <t>Securely store pending upload evidence</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F40" s="45" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>Boveda con contrasena, nada pasa por la galeria. D5 abierta (choca con la revocacion granular).</t>
+        </is>
+      </c>
+      <c r="H40" s="45" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I40" s="5" t="inlineStr">
+        <is>
+          <t>Evidencia cifrada en EvidenceStore, fuera de la galeria.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="40" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="41" t="inlineStr">
+        <is>
+          <t>Evidence Upload / Ingest</t>
+        </is>
+      </c>
+      <c r="C41" s="40" t="inlineStr">
+        <is>
+          <t>Authenticate uploader/device/session and securely transfer evidence</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F41" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>Subida autenticada con el token de sesion (alcance video.upload), verificada el 18-sep. 25-sep (sin probar): corregido que los reintentos perdian incident_id, sha256_plain y media_type (datos en &lt;fev&gt;.evidence.json).</t>
+        </is>
+      </c>
+      <c r="H41" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="I41" s="5" t="inlineStr">
+        <is>
+          <t>25-sep (sin probar): sube con el token prestado por el telefono en vez de 'stub-token', y reanuda lo pendiente al recibirlo. Cancelar/reencolar desde el movil (20-sep) sin probar con hardware.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="40" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="41" t="inlineStr">
+        <is>
+          <t>Upload Integrity Verification</t>
+        </is>
+      </c>
+      <c r="C42" s="40" t="inlineStr">
+        <is>
+          <t>Verify hash, signature, certificate chain and metadata</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F42" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>Verificacion en el servidor.</t>
+        </is>
+      </c>
+      <c r="H42" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="I42" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="40" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="41" t="inlineStr">
+        <is>
+          <t>Evidence Provenance / Chain of Custody</t>
+        </is>
+      </c>
+      <c r="C43" s="40" t="inlineStr">
+        <is>
+          <t>Record who/device/app/session created, transferred or accessed evidence</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F43" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>Manifiesto, linea de tiempo, hashes y diario de auditoria local. Falta el manifiesto formal firmado y registrar quien accede en el backend.</t>
+        </is>
+      </c>
+      <c r="H43" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="I43" s="5" t="inlineStr">
+        <is>
+          <t>25-sep: el manifiesto lleva el agente de la atadura firmada (no uno fijo). Sin registro de accesos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="40" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="41" t="inlineStr">
+        <is>
+          <t>Interrupted Upload / Resume</t>
+        </is>
+      </c>
+      <c r="C44" s="40" t="inlineStr">
+        <is>
+          <t>Safely resume large video uploads without duplication/corruption</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F44" s="45" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="G44" s="5" t="inlineStr">
+        <is>
+          <t>Reanudacion por offset HEAD/PATCH; probada contra el backend local el 18-sep.</t>
+        </is>
+      </c>
+      <c r="H44" s="45" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="I44" s="5" t="inlineStr">
+        <is>
+          <t>ChunkedUploader + UploadSessions con reanudacion; la cola no se rinde nunca.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="40" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="41" t="inlineStr">
+        <is>
+          <t>Evidence Server Acceptance</t>
+        </is>
+      </c>
+      <c r="C45" s="40" t="inlineStr">
+        <is>
+          <t>Backend validates and formally accepts artefact into evidence store</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F45" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>El backend confirma el hash, pero el recibo lo escribe el telefono.</t>
+        </is>
+      </c>
+      <c r="H45" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="I45" s="5" t="inlineStr">
+        <is>
+          <t>Recibo upload.json escrito por la unidad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="40" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="41" t="inlineStr">
+        <is>
+          <t>Local Evidence Deletion</t>
+        </is>
+      </c>
+      <c r="C46" s="40" t="inlineStr">
+        <is>
+          <t>Delete local copy only after verified server acceptance/policy</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F46" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>Se borra tras el recibo local; falta politica y recibo del servidor.</t>
+        </is>
+      </c>
+      <c r="H46" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="I46" s="5" t="inlineStr">
+        <is>
+          <t>Borra el proxy entregado si el servidor no contradice su hash; sin politica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="40" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="41" t="inlineStr">
+        <is>
+          <t>Evidence Access / Playback</t>
+        </is>
+      </c>
+      <c r="C47" s="40" t="inlineStr">
+        <is>
+          <t>Authenticate and authorize viewing</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F47" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>Visionado dentro de la app con contrasena y evento EVIDENCIA_VISUALIZADA en la auditoria. Falta el permiso por politica.</t>
+        </is>
+      </c>
+      <c r="H47" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="I47" s="5" t="inlineStr">
+        <is>
+          <t>La unidad no reproduce evidencia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="40" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="41" t="inlineStr">
+        <is>
+          <t>Evidence Export / Sharing</t>
+        </is>
+      </c>
+      <c r="C48" s="40" t="inlineStr">
+        <is>
+          <t>Controlled export with custody/audit information</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F48" s="46" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>Nada.</t>
+        </is>
+      </c>
+      <c r="H48" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="I48" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="40" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="41" t="inlineStr">
+        <is>
+          <t>Evidence Retention / Archival</t>
+        </is>
+      </c>
+      <c r="C49" s="40" t="inlineStr">
+        <is>
+          <t>Apply tenant/legal retention policy</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F49" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>Politica del tenant.</t>
+        </is>
+      </c>
+      <c r="H49" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="I49" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="40" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="41" t="inlineStr">
+        <is>
+          <t>Evidence Secure Deletion</t>
+        </is>
+      </c>
+      <c r="C50" s="40" t="inlineStr">
+        <is>
+          <t>Controlled destruction following expiry/authorization</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F50" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>Borrado local sin autorizacion ni auditoria.</t>
+        </is>
+      </c>
+      <c r="H50" s="46" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="I50" s="5" t="inlineStr">
+        <is>
+          <t>Nada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="40" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="41" t="inlineStr">
+        <is>
+          <t>Offline Authentication</t>
+        </is>
+      </c>
+      <c r="C51" s="40" t="inlineStr">
+        <is>
+          <t>Permit defined operations when backend cannot be reached</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F51" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>La sesion distingue SOLO_LOCAL de ACREDITADA y desde el 25-sep pasa sola de una a otra al volver la red; falta el permiso offline firmado y su caducidad.</t>
+        </is>
+      </c>
+      <c r="H51" s="46" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="I51" s="5" t="inlineStr">
+        <is>
+          <t>Nada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="40" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="41" t="inlineStr">
+        <is>
+          <t>Offline Recording</t>
+        </is>
+      </c>
+      <c r="C52" s="40" t="inlineStr">
+        <is>
+          <t>Continue evidence creation with cached authorization</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F52" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>Todo funciona offline pero sin gobernar.</t>
+        </is>
+      </c>
+      <c r="H52" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="I52" s="5" t="inlineStr">
+        <is>
+          <t>Graba siempre offline, sin gobernar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="40" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="41" t="inlineStr">
+        <is>
+          <t>Offline → Online Reconciliation</t>
+        </is>
+      </c>
+      <c r="C53" s="40" t="inlineStr">
+        <is>
+          <t>Revalidate identity/bindings and synchronize audit/evidence</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F53" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="G53" s="5" t="inlineStr">
+        <is>
+          <t>Al acreditarse (o renovarse) la sesion sale lo pendiente, ya con su incidente (arreglo del 25-sep, sin probar). Falta revalidar bindings y cuarentena.</t>
+        </is>
+      </c>
+      <c r="H53" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="I53" s="5" t="inlineStr">
+        <is>
+          <t>Reencola lo no entregado en cada arranque y, desde el 25-sep, al recibir token.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="40" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="41" t="inlineStr">
+        <is>
+          <t>Certificate Expiry Handling</t>
+        </is>
+      </c>
+      <c r="C54" s="40" t="inlineStr">
+        <is>
+          <t>Define behaviour when cert expires while device is offline/in operation</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F54" s="46" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
+          <t>Nada.</t>
+        </is>
+      </c>
+      <c r="H54" s="46" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="I54" s="5" t="inlineStr">
+        <is>
+          <t>Nada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="40" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="41" t="inlineStr">
+        <is>
+          <t>Key Rotation</t>
+        </is>
+      </c>
+      <c r="C55" s="40" t="inlineStr">
+        <is>
+          <t>Periodically replace cryptographic keys independently of identity</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F55" s="46" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
+          <t>Nada.</t>
+        </is>
+      </c>
+      <c r="H55" s="46" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="I55" s="5" t="inlineStr">
+        <is>
+          <t>Nada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="40" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="41" t="inlineStr">
+        <is>
+          <t>Key Compromise Recovery</t>
+        </is>
+      </c>
+      <c r="C56" s="40" t="inlineStr">
+        <is>
+          <t>Revoke affected key/cert and establish fresh trust</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F56" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="G56" s="5" t="inlineStr">
+        <is>
+          <t>PKI.</t>
+        </is>
+      </c>
+      <c r="H56" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="I56" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="40" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="41" t="inlineStr">
+        <is>
+          <t>CA / Intermediate CA Rotation</t>
+        </is>
+      </c>
+      <c r="C57" s="40" t="inlineStr">
+        <is>
+          <t>Replace AeriaOne/QPD CA infrastructure without breaking fleet</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F57" s="46" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="G57" s="5" t="inlineStr">
+        <is>
+          <t>Nada: el ancla de perifericos sigue siendo la CA de pruebas.</t>
+        </is>
+      </c>
+      <c r="H57" s="46" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="I57" s="5" t="inlineStr">
+        <is>
+          <t>Nada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="40" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="41" t="inlineStr">
+        <is>
+          <t>Backend Service Identity</t>
+        </is>
+      </c>
+      <c r="C58" s="40" t="inlineStr">
+        <is>
+          <t>Authenticate APIs, upload services, evidence services, etc.</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F58" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="G58" s="5" t="inlineStr">
+        <is>
+          <t>Es del backend. Ojo: hoy se habla en http por el tunel adb, sin TLS ni pinning.</t>
+        </is>
+      </c>
+      <c r="H58" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="I58" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="40" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="41" t="inlineStr">
+        <is>
+          <t>Admin Authentication</t>
+        </is>
+      </c>
+      <c r="C59" s="40" t="inlineStr">
+        <is>
+          <t>Strongly authenticate AeriaOne/QPD administrators</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F59" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="G59" s="5" t="inlineStr">
+        <is>
+          <t>Portal de administracion.</t>
+        </is>
+      </c>
+      <c r="H59" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="I59" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="40" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="41" t="inlineStr">
+        <is>
+          <t>Role / Entitlement Change</t>
+        </is>
+      </c>
+      <c r="C60" s="40" t="inlineStr">
+        <is>
+          <t>Change officer permissions without replacing identity certificate</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F60" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="G60" s="5" t="inlineStr">
+        <is>
+          <t>Portal de administracion.</t>
+        </is>
+      </c>
+      <c r="H60" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="I60" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="40" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="41" t="inlineStr">
+        <is>
+          <t>Emergency Access Revocation</t>
+        </is>
+      </c>
+      <c r="C61" s="40" t="inlineStr">
+        <is>
+          <t>Immediately kill user/device/app/session access</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F61" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="G61" s="5" t="inlineStr">
+        <is>
+          <t>Los 9 interruptores del §13 modelados en TrustState; falta el canal que los entrega.</t>
+        </is>
+      </c>
+      <c r="H61" s="46" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="I61" s="5" t="inlineStr">
+        <is>
+          <t>Nada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="40" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="41" t="inlineStr">
+        <is>
+          <t>Audit Event Generation</t>
+        </is>
+      </c>
+      <c r="C62" s="40" t="inlineStr">
+        <is>
+          <t>Record security-relevant lifecycle events</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F62" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="G62" s="5" t="inlineStr">
+        <is>
+          <t>Diario local encadenado con HMAC (data/audit/), eventos SESION_ACREDITADA / NO_ACREDITADA nuevos. Falta subirlo y ratificar el catalogo.</t>
+        </is>
+      </c>
+      <c r="H62" s="46" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="I62" s="5" t="inlineStr">
+        <is>
+          <t>Ningun diario de auditoria en la unidad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="40" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="41" t="inlineStr">
+        <is>
+          <t>Security Alerting</t>
+        </is>
+      </c>
+      <c r="C63" s="40" t="inlineStr">
+        <is>
+          <t>Detect repeated auth failures, revoked certificates, rogue APK/device, etc.</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F63" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="G63" s="5" t="inlineStr">
+        <is>
+          <t>SIEM.</t>
+        </is>
+      </c>
+      <c r="H63" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="I63" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="40" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" s="41" t="inlineStr">
+        <is>
+          <t>Compromise / Incident Response</t>
+        </is>
+      </c>
+      <c r="C64" s="40" t="inlineStr">
+        <is>
+          <t>Contain compromised user/device/application/key</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F64" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="G64" s="5" t="inlineStr">
+        <is>
+          <t>Respuesta a incidentes.</t>
+        </is>
+      </c>
+      <c r="H64" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="I64" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="40" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" s="41" t="inlineStr">
+        <is>
+          <t>Time Synchronization / Trusted Timestamping</t>
+        </is>
+      </c>
+      <c r="C65" s="40" t="inlineStr">
+        <is>
+          <t>Establish reliable time for signatures, recordings and custody</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F65" s="46" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="G65" s="5" t="inlineStr">
+        <is>
+          <t>Nada (el diario guarda uptime para detectar saltos, pero no hay hora fiable).</t>
+        </is>
+      </c>
+      <c r="H65" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="I65" s="5" t="inlineStr">
+        <is>
+          <t>Device owner: DISALLOW_CONFIG_DATE_TIME y tools/kiosco.sh hora (setTime). No es hora fiable, pero el agente ya no puede tocarla. Sin verificar si el firmware la repone al reiniciar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="40" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="41" t="inlineStr">
+        <is>
+          <t>Backend Trust / Policy Update</t>
+        </is>
+      </c>
+      <c r="C66" s="40" t="inlineStr">
+        <is>
+          <t>Push revocation lists, trust anchors, policies and configuration</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F66" s="46" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="G66" s="5" t="inlineStr">
+        <is>
+          <t>Nada.</t>
+        </is>
+      </c>
+      <c r="H66" s="46" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="I66" s="5" t="inlineStr">
+        <is>
+          <t>Nada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="40" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" s="41" t="inlineStr">
+        <is>
+          <t>Factory Reset / Re-enrollment</t>
+        </is>
+      </c>
+      <c r="C67" s="40" t="inlineStr">
+        <is>
+          <t>Prevent reset device from silently retaining previous identity</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F67" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="G67" s="5" t="inlineStr">
+        <is>
+          <t>deshacerAlta() borra carpetas y claves; falta detectar un reseteo de fabrica y exigir alta nueva.</t>
+        </is>
+      </c>
+      <c r="H67" s="50" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="I67" s="5" t="inlineStr">
+        <is>
+          <t>Device owner con DISALLOW_FACTORY_RESET: impide el reseteo en vez de detectarlo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="40" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="41" t="inlineStr">
+        <is>
+          <t>Return-to-Service</t>
+        </is>
+      </c>
+      <c r="C68" s="40" t="inlineStr">
+        <is>
+          <t>Revalidate repaired/recovered device before restoring trust</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F68" s="46" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="G68" s="5" t="inlineStr">
+        <is>
+          <t>Nada.</t>
+        </is>
+      </c>
+      <c r="H68" s="46" t="inlineStr">
+        <is>
+          <t>Sin empezar</t>
+        </is>
+      </c>
+      <c r="I68" s="5" t="inlineStr">
+        <is>
+          <t>Nada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="40" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" s="41" t="inlineStr">
+        <is>
+          <t>Tenant Transfer / Organizational Reassignment</t>
+        </is>
+      </c>
+      <c r="C69" s="40" t="inlineStr">
+        <is>
+          <t>Safely move asset/person between departments/units where permitted</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="F69" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="G69" s="5" t="inlineStr">
+        <is>
+          <t>Portal de administracion.</t>
+        </is>
+      </c>
+      <c r="H69" s="42" t="inlineStr">
+        <is>
+          <t>No aplica</t>
+        </is>
+      </c>
+      <c r="I69" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="2">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="002E75B6"/>
@@ -6042,7 +9706,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="002E75B6"/>
@@ -11596,7 +15260,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00548235"/>
@@ -12221,7 +15885,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00C00000"/>
@@ -13051,7 +16715,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="007030A0"/>
@@ -14447,7 +18111,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00BF8F00"/>
@@ -14966,7 +18630,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00ED7D31"/>
@@ -15339,634 +19003,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="00ED7D31"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E26"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="62" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="74" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="20" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Trazabilidad de los requisitos IAM-01 a IAM-20</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="26" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Apartado 15 del documento de arquitectura, contrastado contra el codigo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="8" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B4" s="8" t="inlineStr">
-        <is>
-          <t>Requisito</t>
-        </is>
-      </c>
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>Cobertura hoy</t>
-        </is>
-      </c>
-      <c r="D4" s="8" t="inlineStr">
-        <is>
-          <t>Workflows implicados</t>
-        </is>
-      </c>
-      <c r="E4" s="8" t="inlineStr">
-        <is>
-          <t>Nota</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="15" t="inlineStr">
-        <is>
-          <t>IAM-01</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t>Identidad unica y autoritativa para tenant, usuario, dispositivo, credencial, release, instancia de APK, workload, sesion y evidencia</t>
-        </is>
-      </c>
-      <c r="C5" s="11" t="inlineStr">
-        <is>
-          <t>Parcial</t>
-        </is>
-      </c>
-      <c r="D5" s="10" t="inlineStr">
-        <is>
-          <t>12, 23, 36</t>
-        </is>
-      </c>
-      <c r="E5" s="10" t="inlineStr">
-        <is>
-          <t>Dispositivo: si, DEV-8DB2C628 real. Instancia de APK: valor de demo. Evidencia: hay identificador, falta manifiesto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="15" t="inlineStr">
-        <is>
-          <t>IAM-02</t>
-        </is>
-      </c>
-      <c r="B6" s="10" t="inlineStr">
-        <is>
-          <t>Datos, politica y administracion de QPD aislados de otros tenants</t>
-        </is>
-      </c>
-      <c r="C6" s="12" t="inlineStr">
-        <is>
-          <t>No aplica</t>
-        </is>
-      </c>
-      <c r="D6" s="10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E6" s="10" t="inlineStr">
-        <is>
-          <t>Backend.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="15" t="inlineStr">
-        <is>
-          <t>IAM-03</t>
-        </is>
-      </c>
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t>El acceso rutinario recupera el usuario ya enlazado y usa la clave protegida autorizada por PIN</t>
-        </is>
-      </c>
-      <c r="C7" s="11" t="inlineStr">
-        <is>
-          <t>Parcial</t>
-        </is>
-      </c>
-      <c r="D7" s="10" t="inlineStr">
-        <is>
-          <t>4, 27</t>
-        </is>
-      </c>
-      <c r="E7" s="10" t="inlineStr">
-        <is>
-          <t>La pantalla NO pide usuario y el PIN autoriza de verdad el uso de la clave: sin el, firmar como el agente es un error de programacion y no una posibilidad. Lo que falta es que esa autorizacion sea del KEYSTORE y no de la app, que es la decision D2.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="15" t="inlineStr">
-        <is>
-          <t>IAM-04</t>
-        </is>
-      </c>
-      <c r="B8" s="10" t="inlineStr">
-        <is>
-          <t>Reto-respuesta fresco; ni el PIN ni la clave privada se transmiten</t>
-        </is>
-      </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>Cumplido en el cliente</t>
-        </is>
-      </c>
-      <c r="D8" s="10" t="inlineStr">
-        <is>
-          <t>12, 3, 27</t>
-        </is>
-      </c>
-      <c r="E8" s="10" t="inlineStr">
-        <is>
-          <t>La clave nunca sale del Keystore y el PIN tampoco viaja. Desde el 2026-09-06 los cinco puntos que firman usan un nonce ajeno, de un solo uso y con caducidad, verificado con openssl; repetir una respuesta se rechaza. Lo unico que falta para cumplirlo del todo no es del cliente: que el emisor sea un backend y no tools/reto.sh.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="15" t="inlineStr">
-        <is>
-          <t>IAM-05</t>
-        </is>
-      </c>
-      <c r="B9" s="10" t="inlineStr">
-        <is>
-          <t>Claves separadas por proposito e independientemente revocables para usuario, dispositivo, aplicacion y evidencia</t>
-        </is>
-      </c>
-      <c r="C9" s="11" t="inlineStr">
-        <is>
-          <t>Parcial</t>
-        </is>
-      </c>
-      <c r="D9" s="10" t="inlineStr">
-        <is>
-          <t>3, 12, 37, 38</t>
-        </is>
-      </c>
-      <c r="E9" s="10" t="inlineStr">
-        <is>
-          <t>Dispositivo y evidencia ya estan separadas. Falta la del agente (wf 3) y la de firma de evidencia.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="15" t="inlineStr">
-        <is>
-          <t>IAM-06</t>
-        </is>
-      </c>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t>El registro de relaciones es autoritativo para las relaciones y su historia</t>
-        </is>
-      </c>
-      <c r="C10" s="11" t="inlineStr">
-        <is>
-          <t>Parcial</t>
-        </is>
-      </c>
-      <c r="D10" s="10" t="inlineStr">
-        <is>
-          <t>23, 33, 34</t>
-        </is>
-      </c>
-      <c r="E10" s="10" t="inlineStr">
-        <is>
-          <t>El registro autoritativo es del backend y no existe. Lo que si hay desde el 2026-09-06 es la relacion agente-periferico como declaracion firmada con caducidad, que es la mitad que se puede sostener desde el cliente. Falta la atadura agente-telefono registrada (wf 23) y toda la historia de las relaciones.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="15" t="inlineStr">
-        <is>
-          <t>IAM-07</t>
-        </is>
-      </c>
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t>Solo releases aprobados e instancias activas y enlazadas llegan a produccion</t>
-        </is>
-      </c>
-      <c r="C11" s="12" t="inlineStr">
-        <is>
-          <t>Sin empezar</t>
-        </is>
-      </c>
-      <c r="D11" s="10" t="inlineStr">
-        <is>
-          <t>21, 22, 23, 25</t>
-        </is>
-      </c>
-      <c r="E11" s="10" t="inlineStr">
-        <is>
-          <t>Hoy cualquier APK instalado arranca.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="15" t="inlineStr">
-        <is>
-          <t>IAM-08</t>
-        </is>
-      </c>
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t>La autorizacion evalua tenant, sujeto, dispositivos, software, bindings, permisos, recurso, accion y contexto</t>
-        </is>
-      </c>
-      <c r="C12" s="12" t="inlineStr">
-        <is>
-          <t>Sin empezar</t>
-        </is>
-      </c>
-      <c r="D12" s="10" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="E12" s="10" t="inlineStr">
-        <is>
-          <t>Backend. El cliente aun decide en local.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="15" t="inlineStr">
-        <is>
-          <t>IAM-09</t>
-        </is>
-      </c>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>Sesiones cortas, con alcance, identificables y terminables</t>
-        </is>
-      </c>
-      <c r="C13" s="12" t="inlineStr">
-        <is>
-          <t>Sin empezar</t>
-        </is>
-      </c>
-      <c r="D13" s="10" t="inlineStr">
-        <is>
-          <t>28, 29, 30</t>
-        </is>
-      </c>
-      <c r="E13" s="10" t="inlineStr">
-        <is>
-          <t>No hay token de sesion.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="15" t="inlineStr">
-        <is>
-          <t>IAM-10</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>Los perifericos mantienen identidad propia y nunca suplantan al agente</t>
-        </is>
-      </c>
-      <c r="C14" s="11" t="inlineStr">
-        <is>
-          <t>Parcial</t>
-        </is>
-      </c>
-      <c r="D14" s="10" t="inlineStr">
-        <is>
-          <t>13, 31, 33</t>
-        </is>
-      </c>
-      <c r="E14" s="10" t="inlineStr">
-        <is>
-          <t>Verificado sobre hardware el 2026-09-06: la W1 tiene par de claves propio en su Keystore (BWC-896E) y el canal lleva reto-respuesta mutuo. La camara es un tercer sujeto de confianza que se revoca por su lado, no una extension del telefono. Falta el binding agente-camara con caducidad (wf 33).</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="15" t="inlineStr">
-        <is>
-          <t>IAM-11</t>
-        </is>
-      </c>
-      <c r="B15" s="10" t="inlineStr">
-        <is>
-          <t>La evidencia tiene procedencia verificable, integridad, cifrado y custodia</t>
-        </is>
-      </c>
-      <c r="C15" s="11" t="inlineStr">
-        <is>
-          <t>Parcial</t>
-        </is>
-      </c>
-      <c r="D15" s="10" t="inlineStr">
-        <is>
-          <t>36, 37, 38, 42</t>
-        </is>
-      </c>
-      <c r="E15" s="10" t="inlineStr">
-        <is>
-          <t>Cifrado y custodia local: hechos. Procedencia y firma: pendientes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="15" t="inlineStr">
-        <is>
-          <t>IAM-12</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="inlineStr">
-        <is>
-          <t>La aceptacion del servidor precede al borrado local controlado por politica</t>
-        </is>
-      </c>
-      <c r="C16" s="11" t="inlineStr">
-        <is>
-          <t>Parcial</t>
-        </is>
-      </c>
-      <c r="D16" s="10" t="inlineStr">
-        <is>
-          <t>44, 45</t>
-        </is>
-      </c>
-      <c r="E16" s="10" t="inlineStr">
-        <is>
-          <t>El recibo lo escribe hoy el propio telefono.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="15" t="inlineStr">
-        <is>
-          <t>IAM-13</t>
-        </is>
-      </c>
-      <c r="B17" s="10" t="inlineStr">
-        <is>
-          <t>La autorizacion offline es firmada, acotada y reconciliada</t>
-        </is>
-      </c>
-      <c r="C17" s="12" t="inlineStr">
-        <is>
-          <t>Sin empezar</t>
-        </is>
-      </c>
-      <c r="D17" s="10" t="inlineStr">
-        <is>
-          <t>50, 51, 52</t>
-        </is>
-      </c>
-      <c r="E17" s="10" t="inlineStr">
-        <is>
-          <t>Hoy todo funciona offline sin gobierno: es el hueco mas grande respecto al modelo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="15" t="inlineStr">
-        <is>
-          <t>IAM-14</t>
-        </is>
-      </c>
-      <c r="B18" s="10" t="inlineStr">
-        <is>
-          <t>Revocacion granular sobre todos los sujetos de confianza</t>
-        </is>
-      </c>
-      <c r="C18" s="11" t="inlineStr">
-        <is>
-          <t>Parcial</t>
-        </is>
-      </c>
-      <c r="D18" s="10" t="inlineStr">
-        <is>
-          <t>8, 16, 26, 60</t>
-        </is>
-      </c>
-      <c r="E18" s="10" t="inlineStr">
-        <is>
-          <t>Los 9 interruptores del §13 estan modelados en TrustBlockReason; falta el canal. Choca con la boveda (D5).</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="15" t="inlineStr">
-        <is>
-          <t>IAM-15</t>
-        </is>
-      </c>
-      <c r="B19" s="10" t="inlineStr">
-        <is>
-          <t>La revocacion preserva la atribucion historica del momento de la firma</t>
-        </is>
-      </c>
-      <c r="C19" s="12" t="inlineStr">
-        <is>
-          <t>Sin empezar</t>
-        </is>
-      </c>
-      <c r="D19" s="10" t="inlineStr">
-        <is>
-          <t>42</t>
-        </is>
-      </c>
-      <c r="E19" s="10" t="inlineStr">
-        <is>
-          <t>Requiere firma de evidencia (wf 37).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="15" t="inlineStr">
-        <is>
-          <t>IAM-16</t>
-        </is>
-      </c>
-      <c r="B20" s="10" t="inlineStr">
-        <is>
-          <t>Eventos de seguridad, administracion, autorizacion y evidencia correlados y a prueba de manipulacion</t>
-        </is>
-      </c>
-      <c r="C20" s="12" t="inlineStr">
-        <is>
-          <t>Parcial</t>
-        </is>
-      </c>
-      <c r="D20" s="10" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="E20" s="10" t="inlineStr">
-        <is>
-          <t>Diario local a prueba de manipulacion desde el 2026-09-15 (wf 61), con eventos de sesion, periferico y evidencia. Falta correlarlo con el servidor, que es del backend.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="15" t="inlineStr">
-        <is>
-          <t>IAM-17</t>
-        </is>
-      </c>
-      <c r="B21" s="10" t="inlineStr">
-        <is>
-          <t>Los workloads del backend usan identidades propias de minimo privilegio</t>
-        </is>
-      </c>
-      <c r="C21" s="12" t="inlineStr">
-        <is>
-          <t>No aplica</t>
-        </is>
-      </c>
-      <c r="D21" s="10" t="inlineStr">
-        <is>
-          <t>57</t>
-        </is>
-      </c>
-      <c r="E21" s="10" t="inlineStr">
-        <is>
-          <t>Backend.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="15" t="inlineStr">
-        <is>
-          <t>IAM-18</t>
-        </is>
-      </c>
-      <c r="B22" s="10" t="inlineStr">
-        <is>
-          <t>Reseteo o reparacion exigen nueva alta y vuelta a servicio</t>
-        </is>
-      </c>
-      <c r="C22" s="11" t="inlineStr">
-        <is>
-          <t>Parcial</t>
-        </is>
-      </c>
-      <c r="D22" s="10" t="inlineStr">
-        <is>
-          <t>66, 67</t>
-        </is>
-      </c>
-      <c r="E22" s="10" t="inlineStr">
-        <is>
-          <t>La clave se destruye con el reseteo, pero no se DETECTA: la app simplemente deja de funcionar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="15" t="inlineStr">
-        <is>
-          <t>IAM-19</t>
-        </is>
-      </c>
-      <c r="B23" s="10" t="inlineStr">
-        <is>
-          <t>La rotacion de CA admite solape controlado y migracion de la flota</t>
-        </is>
-      </c>
-      <c r="C23" s="12" t="inlineStr">
-        <is>
-          <t>Sin empezar</t>
-        </is>
-      </c>
-      <c r="D23" s="10" t="inlineStr">
-        <is>
-          <t>56</t>
-        </is>
-      </c>
-      <c r="E23" s="10" t="inlineStr">
-        <is>
-          <t>Hoy solo hay una CA de pruebas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="15" t="inlineStr">
-        <is>
-          <t>IAM-20</t>
-        </is>
-      </c>
-      <c r="B24" s="10" t="inlineStr">
-        <is>
-          <t>La linea base no reclama biometria ni MFA formal para el agente</t>
-        </is>
-      </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>Cumplido</t>
-        </is>
-      </c>
-      <c r="D24" s="10" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="E24" s="10" t="inlineStr">
-        <is>
-          <t>La app no usa biometria. Coherente por diseno, no por omision.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="20" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B26" s="21" t="inlineStr">
-        <is>
-          <t>20 requisitos</t>
-        </is>
-      </c>
-      <c r="C26" s="21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D26" s="21" t="inlineStr">
-        <is>
-          <t>Cumplido: 1 | Parcial: 9 | Sin empezar: 7 | No aplica (backend): 2</t>
-        </is>
-      </c>
-      <c r="E26" s="21" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>